<commit_message>
Prep for second run of Proposal
</commit_message>
<xml_diff>
--- a/Research Logs/Dave/Research Log - Dave.xlsx
+++ b/Research Logs/Dave/Research Log - Dave.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://w2shared-my.sharepoint.com/personal/dave_sushames01_student_wandw_ac_nz/Documents/Documents/Capstone/Research Logs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://w2shared-my.sharepoint.com/personal/dave_sushames01_student_wandw_ac_nz/Documents/Documents/Capstone/Research Logs/Dave/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="13_ncr:1_{AF0BDED7-A538-4982-BD37-86F9ACE43960}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9AAFDA93-A77D-4277-85B2-39ECBFA78F06}"/>
+  <xr:revisionPtr revIDLastSave="101" documentId="13_ncr:1_{AF0BDED7-A538-4982-BD37-86F9ACE43960}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{70C1E10A-E556-486A-A49A-C54796DDC3DC}"/>
   <bookViews>
-    <workbookView xWindow="3720" yWindow="3180" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="165" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Research template" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="35">
   <si>
     <t>Date</t>
   </si>
@@ -110,6 +110,60 @@
   </si>
   <si>
     <t>Requires BIOS config to determine which card to use</t>
+  </si>
+  <si>
+    <t>Watching</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=gmmPfDCRfrQ</t>
+  </si>
+  <si>
+    <t>How Kanban works, practices</t>
+  </si>
+  <si>
+    <t>Visualise everything. To do/In progress/done boards?</t>
+  </si>
+  <si>
+    <t>Found 3 sources</t>
+  </si>
+  <si>
+    <t>https://www.atlassian.com/agile/kanban</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Found some best practices, what it intends to solve, and </t>
+  </si>
+  <si>
+    <t>https://allthingsagile.co/post/kanban-practices-and-principles/</t>
+  </si>
+  <si>
+    <t>Briefly read, seems to have a lot of info already covered by previous sources</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=rnMToOThBuk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seems for intended for software development/cyclical/iterative approach, which the team has expressed a distaste for. </t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=W94eceurqAQ</t>
+  </si>
+  <si>
+    <t>How to actually get started with Kanban</t>
+  </si>
+  <si>
+    <t>Intended for organisation that already have an existing process and customer base, rather than a new group. Not particularly  useful.</t>
+  </si>
+  <si>
+    <t>Finding AI Digital Forensics tools</t>
+  </si>
+  <si>
+    <t>7 sources found an briefly examined</t>
+  </si>
+  <si>
+    <t>https://aiforensics.org/</t>
+  </si>
+  <si>
+    <t>Is about investigating AI, rather than using AI to investigate. Not useful.</t>
   </si>
 </sst>
 </file>
@@ -171,7 +225,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -180,10 +234,14 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -469,55 +527,55 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:G15"/>
+  <dimension ref="B2:G20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="13.140625" style="3" customWidth="1"/>
     <col min="3" max="4" width="23.85546875" customWidth="1"/>
-    <col min="5" max="5" width="76.140625" customWidth="1"/>
-    <col min="6" max="6" width="52.140625" customWidth="1"/>
+    <col min="5" max="5" width="53.42578125" customWidth="1"/>
+    <col min="6" max="6" width="74.28515625" customWidth="1"/>
     <col min="7" max="7" width="131" customWidth="1"/>
     <col min="8" max="8" width="33.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="5">
+      <c r="D2" s="4">
         <f>ROUNDDOWN(SUM(C7:C500)/60,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="3" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="5">
+      <c r="D3" s="4">
         <f>ROUND(MOD(SUM(C7:C500),60),0)</f>
-        <v>15</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" s="6" t="s">
         <v>6</v>
       </c>
     </row>
@@ -565,12 +623,166 @@
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
     </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B10" s="7">
+        <v>46248</v>
+      </c>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B11" s="7">
+        <v>46248</v>
+      </c>
+      <c r="C11" s="1">
+        <v>5</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B12" s="7">
+        <v>46248</v>
+      </c>
+      <c r="C12" s="1">
+        <v>15</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="13" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B13" s="7">
+        <v>46248</v>
+      </c>
+      <c r="C13" s="1">
+        <v>20</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="F14" s="1"/>
-      <c r="G14" s="2"/>
-    </row>
-    <row r="15" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="F15" s="1"/>
+      <c r="B14" s="7">
+        <v>46248</v>
+      </c>
+      <c r="C14" s="1">
+        <v>5</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="15" spans="2:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="B15" s="7">
+        <v>46248</v>
+      </c>
+      <c r="C15" s="1">
+        <v>15</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="16" spans="2:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="C16" s="1">
+        <v>15</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="G16" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B17" s="3">
+        <v>46251</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C19" s="1">
+        <v>10</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E19" t="s">
+        <v>31</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C20" s="1">
+        <v>5</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G20" t="s">
+        <v>33</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Project plan update, minus AI bit
</commit_message>
<xml_diff>
--- a/Research Logs/Dave/Research Log - Dave.xlsx
+++ b/Research Logs/Dave/Research Log - Dave.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://w2shared-my.sharepoint.com/personal/dave_sushames01_student_wandw_ac_nz/Documents/Documents/Capstone/Research Logs/Dave/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="101" documentId="13_ncr:1_{AF0BDED7-A538-4982-BD37-86F9ACE43960}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{70C1E10A-E556-486A-A49A-C54796DDC3DC}"/>
+  <xr:revisionPtr revIDLastSave="109" documentId="13_ncr:1_{AF0BDED7-A538-4982-BD37-86F9ACE43960}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8925ED19-939A-44BF-AD61-80039C5BD7A7}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="165" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-26940" yWindow="0" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Research template" sheetId="1" r:id="rId1"/>
@@ -160,10 +160,10 @@
     <t>7 sources found an briefly examined</t>
   </si>
   <si>
+    <t>Is about investigating AI, rather than using AI to investigate. Not useful.</t>
+  </si>
+  <si>
     <t>https://aiforensics.org/</t>
-  </si>
-  <si>
-    <t>Is about investigating AI, rather than using AI to investigate. Not useful.</t>
   </si>
 </sst>
 </file>
@@ -173,7 +173,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="d/mm/yy;@"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -193,6 +193,13 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -225,7 +232,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -242,6 +249,13 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -729,6 +743,9 @@
       </c>
     </row>
     <row r="16" spans="2:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="B16" s="3">
+        <v>46248</v>
+      </c>
       <c r="C16" s="1">
         <v>15</v>
       </c>
@@ -745,44 +762,51 @@
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B17" s="3">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B18" s="8">
         <v>46251</v>
       </c>
+      <c r="C18" s="9">
+        <v>10</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E18" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="F18" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="G18" s="9" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C19" s="1">
-        <v>10</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E19" t="s">
-        <v>31</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>10</v>
+      <c r="B19" s="8"/>
+      <c r="C19" s="9">
+        <v>5</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G19" s="10" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C20" s="1">
-        <v>5</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="G20" t="s">
-        <v>33</v>
-      </c>
+      <c r="B20" s="8"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="10"/>
+      <c r="G20" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>